<commit_message>
sync 2026-05-15: content +new/-deleted, collection, multilingual
</commit_message>
<xml_diff>
--- a/reports/content/hi/2026-05-15_sync_report.xlsx
+++ b/reports/content/hi/2026-05-15_sync_report.xlsx
@@ -462,13 +462,13 @@
         <v>0</v>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1247</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="5">
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.3% of prev</t>
+          <t>0.0% of prev</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,567 +695,6 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>after</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>69f87d9e0a2be3f28188f4e7</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>a79e99c8-0efb-4276-8240-5b9f747ffc62</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>sentence</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">चित्र में कौन सो रहा है? </t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>69f87d9e8639790c76fd864a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>c7f7a8e7-8da1-4217-a1c0-515dcd3ec62f</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>sentence</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">चित्र में कौन सा मौसम है? </t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>69f87d9f40035c0088f198fb</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>8be02bcd-5f6a-4249-ac10-888ebec2876c</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>sentence</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">माला पैर में क्या पहनकर घूमने लगी? </t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>69faddccc5221c5660cd3c94</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>04c1612b-a88e-403d-beed-7e33f6015565</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">सुशीला का जन्मदिन था। वह इसे खास तरीके से मनाना चाहती थी। वो अपने दोस्तों के साथ क्या कर रही है ? </t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>69faddd09c807bc6072aeec2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>b17d7c94-5104-4ef3-b0da-f46d84972733</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">चींटी और हाथी छुपन-छुपाई खेल रहे हैं। चींटी को पता चल जाता है कि हाथी कहाँ छुपा है। चित्र में हाथी कहाँ छुपा है ? </t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>69faddd166837dc8bbc2267e</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2831f37a-d8d0-4304-8a95-d6afdc6dd4fe</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">सर्दी की सुबह थी। बच्चों के स्कूल का वार्षिक दिवस था। सभी बच्चे अपने स्कूल को सजाना चाहते थे। वे सजावट के लिए क्या इकट्ठा कर रहे थे? </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>69faddd1c5221c5660cd3ca4</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>3f129685-d3c2-4655-966b-37a2c500908b</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">यह घटना बादशाह अकबर के दरबार में घटी। एक ग्रामीण मदद मांगने दरबार में आया। बादशाह अकबर ने उस ग्रामीण की मदद कैसे की? </t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>69faddd366837dc8bbc22684</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>bb8c1bf2-dc28-4b19-8a8b-6b881a5293c9</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">एक बिल्ली नींद से जाग उठी। उसे बहुत भूख लगी थी। बिल्ली क्या बना रही है? </t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>69faddd3c5221c5660cd3cae</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>a4b2e14c-35f8-46ed-860f-b7ae6c875e7e</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">एक बगीचे में एक घोंघा रहता था। घोंघे ने अपना सारा जीवन बगीचे में बिताया था। एक दिन उसने सोचा "मैं बाहर जाकर देखूँगा कि दुनिया कैसी है।” घोंघा ने बाहर जाने की कैसी तैयारी की? </t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>69faddd4c5221c5660cd3cb2</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>6336a751-5f64-432c-879a-9056695d6031</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">प्राचीन काल में संदेश भेजने के लिए व्यक्ति होते थे। जिन्हें दूत कहा जाता था। कम दूरी के लिए पैदल ही जाकर पत्र पहुँचा देते थे। लंबी दूरी के लिए किसे भेजे जाते थे ? </t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>69faddd566837dc8bbc2268c</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>457e3eaf-974c-4516-862c-a2c526255f47</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">एक राजा को प्रश्न पूछने में रुचि थी। वह अपने प्रश्नों के माध्यम से मंत्रियों की परीक्षा लेता था। यदि राजा उत्तर से संतुष्ट होता था, तो वह उन्हें उपहार देता था। राजा उपहार में क्या देता था? </t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>69faddd5c5221c5660cd3cb4</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>59d77106-73b3-4ac7-a0f7-eb5016e354b1</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">एक सुहावनी दोपहर थी। रम्या के पास रानी नाम की एक पालतू बिल्ली है। वह बाहर दौड़ने जाना चाहती थी। रम्या क्या करने की कोशिश कर रही है? </t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>69faddd79c807bc6072aeede</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>76889172-bcf3-4362-804a-938923bf19e0</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">एक राजा अपने न्याय और विवेक के लिए बहुत प्रसिद्ध थे। एक दिन उसे एक सपना आया। एक मूर्ती अपने पंक फैलाकर आकाश में उड़ रही थी। उस मूर्ती के हाथ में क्या था? </t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>69faddd8245ea0aba052b844</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>e092fb2f-0e43-41c0-b31b-72a45a283836</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">भवानी, प्रसाद और मिश्रा नाचते, गाते झूमने लगे। वे त्यौहार के दिन बहुत खुश थे। चारों ओर रंग ही रंग था। वे कौनसा त्यौहार मना रहे थे ? </t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>69faddda66837dc8bbc226a2</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>df20ca84-1075-4db3-bc7e-215777c41b71</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">चिन्नू और चिंटू सरकारी स्कूल जाते हैं। वहा सहायता, समझदारी और अच्छे कर्मों के बारे में सिखाते हैं। वे इन्हें वास्तविक जीवन में लागू करने का प्रयास करते हैं। चित्र में चिन्नू और चिंटू क्या कर रहे है? </t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>69fadddc245ea0aba052b852</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>4641d00d-56c5-4e05-b3c5-71524b5e84cc</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">सड़क पर चलते समय सावधानी बरतें। सड़क के किनारे बनी पटरियों का उपयोग करें। यातायात संकेतक नियमों का पालन करें। जब लाल बत्ती जलती है, तब हमें क्या करनी चाहिए ? </t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>69fadddc9c807bc6072aeeec</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>08d7b336-44d7-4c07-b37b-4c1a970614c9</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>paragraph</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">वेंकट तमिलनाडु का रहने वाला है। वह तमिल भाषा बोलता है। खाने में उसे इडली सांभर पसंद है। वेंकट खाना किस में खता है ? </t>
         </is>
       </c>
     </row>

</xml_diff>